<commit_message>
updates to the pipelines
</commit_message>
<xml_diff>
--- a/docs/resources/SampleSheet.xlsx
+++ b/docs/resources/SampleSheet.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="78">
   <si>
     <t>PCR A</t>
   </si>
@@ -253,6 +253,24 @@
   </si>
   <si>
     <t>RV2 VALUES</t>
+  </si>
+  <si>
+    <t>Idx_Fw1_7</t>
+  </si>
+  <si>
+    <t>Idx_Fw1_8</t>
+  </si>
+  <si>
+    <t>Idx_Rv1_5</t>
+  </si>
+  <si>
+    <t>Idx_Rv1_6</t>
+  </si>
+  <si>
+    <t>Idx_Rv2_5</t>
+  </si>
+  <si>
+    <t>Idx_Rv2_6</t>
   </si>
 </sst>
 </file>
@@ -1158,19 +1176,19 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" showInputMessage="1" showErrorMessage="1" xr:uid="{6C0CB346-6BDF-3A44-AE97-FD406DDA2749}">
           <x14:formula1>
-            <xm:f>'List Values'!$A$2:$A$8</xm:f>
+            <xm:f>'List Values'!$A$2:$A$9</xm:f>
           </x14:formula1>
           <xm:sqref>B3:B26 D3:D26</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3888EA7F-674D-3643-A2AD-311ED4D278A8}">
           <x14:formula1>
-            <xm:f>'List Values'!$B$2:$B$6</xm:f>
+            <xm:f>'List Values'!$B$2:$B$7</xm:f>
           </x14:formula1>
           <xm:sqref>C3:C26</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{22BE3218-B310-9E4C-828A-41D38887CF01}">
           <x14:formula1>
-            <xm:f>'List Values'!$C$2:$C$6</xm:f>
+            <xm:f>'List Values'!$C$2:$C$7</xm:f>
           </x14:formula1>
           <xm:sqref>E3:E26</xm:sqref>
         </x14:dataValidation>
@@ -1182,7 +1200,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{65416F45-D3E4-7B46-8008-C00D4B238C92}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
     <col min="1" max="1" width="25.375" customWidth="1"/>
@@ -1249,10 +1267,32 @@
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="B6" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="2" t="s">
         <v>25</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="1" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>